<commit_message>
Plantillas 4.1/4.2: S1-00334 solo admite systemDiffCode A
El objectValue F ("solo los DM del BREX S1000D/ATA") dejaba pasar F en
cualquier data module, así que un ejemplo de rechazo correcto ("F en un
DM normal") salía aceptado. En las dos plantillas la regla queda solo con
valueAllowed="A", objectUse "must be 'A'; no UOC is used." y Proposal
"No need for SDC seen, use default A.". Solo cambian las celdas Proposal
y Rule de esa fila (comprobado celda a celda con HEAD, valor y estilo).

Tabla del motor (F pasa a romper la regla), simulador y los dos casos
del juego de pruebas actualizados. Lint de plantillas: 0 hallazgos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rwcp9cSck72V1zULNhL8wU
</commit_message>
<xml_diff>
--- a/public/brdp-template-4-1.xlsx
+++ b/public/brdp-template-4-1.xlsx
@@ -644,7 +644,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>No need for SDC seen, use default. SDC to be used if different LRUs are in identical SNS.</t>
+          <t>No need for SDC seen, use default A.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -661,9 +661,8 @@
         <is>
           <t>&lt;structureObjectRule&gt;
   &lt;objectPath allowedObjectFlag="2"&gt;//@systemDiffCode&lt;/objectPath&gt;
-  &lt;objectUse&gt;BRDP-S1-00334. The system difference code (@systemDiffCode) should be 'A', used only when different LRUs share an identical SNS; no UOC is used.&lt;/objectUse&gt;
+  &lt;objectUse&gt;BRDP-S1-00334. The system difference code (@systemDiffCode) must be 'A'; no UOC is used.&lt;/objectUse&gt;
   &lt;objectValue valueForm="single" valueAllowed="A"&gt;SDC to be used if different LRUs are in identical SNS. No UOC is used.&lt;/objectValue&gt;
-  &lt;objectValue valueForm="single" valueAllowed="F"&gt;Only the S1000D and ATA BREX data modules use systemDiffCode F.&lt;/objectValue&gt;
 &lt;/structureObjectRule&gt;</t>
         </is>
       </c>

</xml_diff>